<commit_message>
chore(telemetry): sync 346 verified backlinks, multi-protocol indexing logs, and edge telemetry
</commit_message>
<xml_diff>
--- a/reports/MASTER_LIVE_BACKLINKS_REPORT.xlsx
+++ b/reports/MASTER_LIVE_BACKLINKS_REPORT.xlsx
@@ -596,7 +596,7 @@
         </is>
       </c>
       <c r="I2" s="2" t="n">
-        <v>1004</v>
+        <v>879</v>
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
@@ -647,7 +647,7 @@
         </is>
       </c>
       <c r="I3" s="2" t="n">
-        <v>1083</v>
+        <v>1158</v>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
@@ -698,7 +698,7 @@
         </is>
       </c>
       <c r="I4" s="2" t="n">
-        <v>394</v>
+        <v>497</v>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="I5" s="2" t="n">
-        <v>290</v>
+        <v>640</v>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
@@ -800,7 +800,7 @@
         </is>
       </c>
       <c r="I6" s="2" t="n">
-        <v>458</v>
+        <v>390</v>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="I7" s="2" t="n">
-        <v>299</v>
+        <v>373</v>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
@@ -902,7 +902,7 @@
         </is>
       </c>
       <c r="I8" s="2" t="n">
-        <v>1075</v>
+        <v>825</v>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
@@ -953,7 +953,7 @@
         </is>
       </c>
       <c r="I9" s="2" t="n">
-        <v>909</v>
+        <v>801</v>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
@@ -1004,7 +1004,7 @@
         </is>
       </c>
       <c r="I10" s="2" t="n">
-        <v>1161</v>
+        <v>903</v>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
@@ -1055,7 +1055,7 @@
         </is>
       </c>
       <c r="I11" s="2" t="n">
-        <v>848</v>
+        <v>873</v>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
@@ -1106,7 +1106,7 @@
         </is>
       </c>
       <c r="I12" s="2" t="n">
-        <v>892</v>
+        <v>850</v>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="I13" s="2" t="n">
-        <v>796</v>
+        <v>904</v>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
@@ -1208,7 +1208,7 @@
         </is>
       </c>
       <c r="I14" s="2" t="n">
-        <v>838</v>
+        <v>964</v>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
@@ -1259,7 +1259,7 @@
         </is>
       </c>
       <c r="I15" s="2" t="n">
-        <v>821</v>
+        <v>841</v>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
@@ -1310,7 +1310,7 @@
         </is>
       </c>
       <c r="I16" s="2" t="n">
-        <v>778</v>
+        <v>861</v>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
@@ -1361,7 +1361,7 @@
         </is>
       </c>
       <c r="I17" s="2" t="n">
-        <v>853</v>
+        <v>973</v>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
@@ -1412,7 +1412,7 @@
         </is>
       </c>
       <c r="I18" s="2" t="n">
-        <v>886</v>
+        <v>979</v>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
@@ -1463,7 +1463,7 @@
         </is>
       </c>
       <c r="I19" s="2" t="n">
-        <v>843</v>
+        <v>877</v>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
@@ -1514,7 +1514,7 @@
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>817</v>
+        <v>972</v>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
@@ -1565,7 +1565,7 @@
         </is>
       </c>
       <c r="I21" s="2" t="n">
-        <v>916</v>
+        <v>819</v>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
@@ -1616,7 +1616,7 @@
         </is>
       </c>
       <c r="I22" s="2" t="n">
-        <v>833</v>
+        <v>874</v>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
@@ -1667,7 +1667,7 @@
         </is>
       </c>
       <c r="I23" s="2" t="n">
-        <v>925</v>
+        <v>812</v>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
@@ -1718,7 +1718,7 @@
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>1289</v>
+        <v>1054</v>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
@@ -1769,7 +1769,7 @@
         </is>
       </c>
       <c r="I25" s="2" t="n">
-        <v>793</v>
+        <v>954</v>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
@@ -1820,7 +1820,7 @@
         </is>
       </c>
       <c r="I26" s="2" t="n">
-        <v>779</v>
+        <v>788</v>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
@@ -1871,7 +1871,7 @@
         </is>
       </c>
       <c r="I27" s="2" t="n">
-        <v>778</v>
+        <v>805</v>
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
@@ -1922,7 +1922,7 @@
         </is>
       </c>
       <c r="I28" s="2" t="n">
-        <v>907</v>
+        <v>856</v>
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
         </is>
       </c>
       <c r="I29" s="2" t="n">
-        <v>814</v>
+        <v>839</v>
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
@@ -2024,7 +2024,7 @@
         </is>
       </c>
       <c r="I30" s="2" t="n">
-        <v>785</v>
+        <v>720</v>
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
@@ -2075,7 +2075,7 @@
         </is>
       </c>
       <c r="I31" s="2" t="n">
-        <v>790</v>
+        <v>742</v>
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
@@ -2126,7 +2126,7 @@
         </is>
       </c>
       <c r="I32" s="2" t="n">
-        <v>693</v>
+        <v>776</v>
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
@@ -2177,7 +2177,7 @@
         </is>
       </c>
       <c r="I33" s="2" t="n">
-        <v>898</v>
+        <v>817</v>
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
@@ -2228,7 +2228,7 @@
         </is>
       </c>
       <c r="I34" s="2" t="n">
-        <v>747</v>
+        <v>963</v>
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
@@ -2279,7 +2279,7 @@
         </is>
       </c>
       <c r="I35" s="2" t="n">
-        <v>723</v>
+        <v>775</v>
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
@@ -2330,7 +2330,7 @@
         </is>
       </c>
       <c r="I36" s="2" t="n">
-        <v>771</v>
+        <v>755</v>
       </c>
       <c r="J36" s="4" t="inlineStr">
         <is>
@@ -2381,7 +2381,7 @@
         </is>
       </c>
       <c r="I37" s="2" t="n">
-        <v>748</v>
+        <v>904</v>
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
@@ -2432,7 +2432,7 @@
         </is>
       </c>
       <c r="I38" s="2" t="n">
-        <v>737</v>
+        <v>773</v>
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
         </is>
       </c>
       <c r="I39" s="2" t="n">
-        <v>816</v>
+        <v>811</v>
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
@@ -2534,7 +2534,7 @@
         </is>
       </c>
       <c r="I40" s="2" t="n">
-        <v>807</v>
+        <v>931</v>
       </c>
       <c r="J40" s="4" t="inlineStr">
         <is>
@@ -2585,7 +2585,7 @@
         </is>
       </c>
       <c r="I41" s="2" t="n">
-        <v>780</v>
+        <v>778</v>
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
@@ -2636,7 +2636,7 @@
         </is>
       </c>
       <c r="I42" s="2" t="n">
-        <v>846</v>
+        <v>814</v>
       </c>
       <c r="J42" s="4" t="inlineStr">
         <is>
@@ -2687,7 +2687,7 @@
         </is>
       </c>
       <c r="I43" s="2" t="n">
-        <v>696</v>
+        <v>759</v>
       </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
@@ -2738,7 +2738,7 @@
         </is>
       </c>
       <c r="I44" s="2" t="n">
-        <v>928</v>
+        <v>786</v>
       </c>
       <c r="J44" s="4" t="inlineStr">
         <is>
@@ -2789,7 +2789,7 @@
         </is>
       </c>
       <c r="I45" s="2" t="n">
-        <v>803</v>
+        <v>805</v>
       </c>
       <c r="J45" s="4" t="inlineStr">
         <is>
@@ -2840,7 +2840,7 @@
         </is>
       </c>
       <c r="I46" s="2" t="n">
-        <v>735</v>
+        <v>772</v>
       </c>
       <c r="J46" s="4" t="inlineStr">
         <is>
@@ -2891,7 +2891,7 @@
         </is>
       </c>
       <c r="I47" s="2" t="n">
-        <v>741</v>
+        <v>757</v>
       </c>
       <c r="J47" s="4" t="inlineStr">
         <is>
@@ -2942,7 +2942,7 @@
         </is>
       </c>
       <c r="I48" s="2" t="n">
-        <v>872</v>
+        <v>786</v>
       </c>
       <c r="J48" s="4" t="inlineStr">
         <is>
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="I49" s="2" t="n">
-        <v>752</v>
+        <v>782</v>
       </c>
       <c r="J49" s="4" t="inlineStr">
         <is>
@@ -3044,7 +3044,7 @@
         </is>
       </c>
       <c r="I50" s="2" t="n">
-        <v>835</v>
+        <v>797</v>
       </c>
       <c r="J50" s="4" t="inlineStr">
         <is>
@@ -3095,7 +3095,7 @@
         </is>
       </c>
       <c r="I51" s="2" t="n">
-        <v>793</v>
+        <v>776</v>
       </c>
       <c r="J51" s="4" t="inlineStr">
         <is>
@@ -3146,7 +3146,7 @@
         </is>
       </c>
       <c r="I52" s="2" t="n">
-        <v>751</v>
+        <v>724</v>
       </c>
       <c r="J52" s="4" t="inlineStr">
         <is>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="I53" s="2" t="n">
-        <v>799</v>
+        <v>767</v>
       </c>
       <c r="J53" s="4" t="inlineStr">
         <is>
@@ -3248,7 +3248,7 @@
         </is>
       </c>
       <c r="I54" s="2" t="n">
-        <v>823</v>
+        <v>757</v>
       </c>
       <c r="J54" s="4" t="inlineStr">
         <is>
@@ -3299,7 +3299,7 @@
         </is>
       </c>
       <c r="I55" s="2" t="n">
-        <v>764</v>
+        <v>754</v>
       </c>
       <c r="J55" s="4" t="inlineStr">
         <is>
@@ -3350,7 +3350,7 @@
         </is>
       </c>
       <c r="I56" s="2" t="n">
-        <v>751</v>
+        <v>732</v>
       </c>
       <c r="J56" s="4" t="inlineStr">
         <is>
@@ -3401,7 +3401,7 @@
         </is>
       </c>
       <c r="I57" s="2" t="n">
-        <v>740</v>
+        <v>735</v>
       </c>
       <c r="J57" s="4" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
         </is>
       </c>
       <c r="I58" s="2" t="n">
-        <v>870</v>
+        <v>780</v>
       </c>
       <c r="J58" s="4" t="inlineStr">
         <is>
@@ -3503,7 +3503,7 @@
         </is>
       </c>
       <c r="I59" s="2" t="n">
-        <v>791</v>
+        <v>807</v>
       </c>
       <c r="J59" s="4" t="inlineStr">
         <is>
@@ -3554,7 +3554,7 @@
         </is>
       </c>
       <c r="I60" s="2" t="n">
-        <v>814</v>
+        <v>732</v>
       </c>
       <c r="J60" s="4" t="inlineStr">
         <is>
@@ -3605,7 +3605,7 @@
         </is>
       </c>
       <c r="I61" s="2" t="n">
-        <v>849</v>
+        <v>796</v>
       </c>
       <c r="J61" s="4" t="inlineStr">
         <is>
@@ -3656,7 +3656,7 @@
         </is>
       </c>
       <c r="I62" s="2" t="n">
-        <v>826</v>
+        <v>830</v>
       </c>
       <c r="J62" s="4" t="inlineStr">
         <is>
@@ -3707,7 +3707,7 @@
         </is>
       </c>
       <c r="I63" s="2" t="n">
-        <v>775</v>
+        <v>738</v>
       </c>
       <c r="J63" s="4" t="inlineStr">
         <is>
@@ -3758,7 +3758,7 @@
         </is>
       </c>
       <c r="I64" s="2" t="n">
-        <v>753</v>
+        <v>722</v>
       </c>
       <c r="J64" s="4" t="inlineStr">
         <is>
@@ -3809,7 +3809,7 @@
         </is>
       </c>
       <c r="I65" s="2" t="n">
-        <v>722</v>
+        <v>1112</v>
       </c>
       <c r="J65" s="4" t="inlineStr">
         <is>
@@ -3860,7 +3860,7 @@
         </is>
       </c>
       <c r="I66" s="2" t="n">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="J66" s="4" t="inlineStr">
         <is>
@@ -3911,7 +3911,7 @@
         </is>
       </c>
       <c r="I67" s="2" t="n">
-        <v>771</v>
+        <v>855</v>
       </c>
       <c r="J67" s="4" t="inlineStr">
         <is>
@@ -3962,7 +3962,7 @@
         </is>
       </c>
       <c r="I68" s="2" t="n">
-        <v>669</v>
+        <v>987</v>
       </c>
       <c r="J68" s="4" t="inlineStr">
         <is>
@@ -4013,7 +4013,7 @@
         </is>
       </c>
       <c r="I69" s="2" t="n">
-        <v>694</v>
+        <v>734</v>
       </c>
       <c r="J69" s="4" t="inlineStr">
         <is>
@@ -4064,7 +4064,7 @@
         </is>
       </c>
       <c r="I70" s="2" t="n">
-        <v>664</v>
+        <v>929</v>
       </c>
       <c r="J70" s="4" t="inlineStr">
         <is>
@@ -4115,7 +4115,7 @@
         </is>
       </c>
       <c r="I71" s="2" t="n">
-        <v>692</v>
+        <v>642</v>
       </c>
       <c r="J71" s="4" t="inlineStr">
         <is>
@@ -4166,7 +4166,7 @@
         </is>
       </c>
       <c r="I72" s="2" t="n">
-        <v>681</v>
+        <v>672</v>
       </c>
       <c r="J72" s="4" t="inlineStr">
         <is>
@@ -4217,7 +4217,7 @@
         </is>
       </c>
       <c r="I73" s="2" t="n">
-        <v>749</v>
+        <v>711</v>
       </c>
       <c r="J73" s="4" t="inlineStr">
         <is>
@@ -4268,7 +4268,7 @@
         </is>
       </c>
       <c r="I74" s="2" t="n">
-        <v>740</v>
+        <v>666</v>
       </c>
       <c r="J74" s="4" t="inlineStr">
         <is>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="I75" s="2" t="n">
-        <v>698</v>
+        <v>693</v>
       </c>
       <c r="J75" s="4" t="inlineStr">
         <is>
@@ -4370,7 +4370,7 @@
         </is>
       </c>
       <c r="I76" s="2" t="n">
-        <v>882</v>
+        <v>710</v>
       </c>
       <c r="J76" s="4" t="inlineStr">
         <is>
@@ -4421,7 +4421,7 @@
         </is>
       </c>
       <c r="I77" s="2" t="n">
-        <v>870</v>
+        <v>732</v>
       </c>
       <c r="J77" s="4" t="inlineStr">
         <is>
@@ -4472,7 +4472,7 @@
         </is>
       </c>
       <c r="I78" s="2" t="n">
-        <v>732</v>
+        <v>695</v>
       </c>
       <c r="J78" s="4" t="inlineStr">
         <is>
@@ -4523,7 +4523,7 @@
         </is>
       </c>
       <c r="I79" s="2" t="n">
-        <v>705</v>
+        <v>640</v>
       </c>
       <c r="J79" s="4" t="inlineStr">
         <is>
@@ -4574,7 +4574,7 @@
         </is>
       </c>
       <c r="I80" s="2" t="n">
-        <v>6872</v>
+        <v>908</v>
       </c>
       <c r="J80" s="4" t="inlineStr">
         <is>
@@ -4625,7 +4625,7 @@
         </is>
       </c>
       <c r="I81" s="2" t="n">
-        <v>732</v>
+        <v>690</v>
       </c>
       <c r="J81" s="4" t="inlineStr">
         <is>
@@ -4676,7 +4676,7 @@
         </is>
       </c>
       <c r="I82" s="2" t="n">
-        <v>718</v>
+        <v>690</v>
       </c>
       <c r="J82" s="4" t="inlineStr">
         <is>
@@ -4727,7 +4727,7 @@
         </is>
       </c>
       <c r="I83" s="2" t="n">
-        <v>686</v>
+        <v>683</v>
       </c>
       <c r="J83" s="4" t="inlineStr">
         <is>
@@ -4778,7 +4778,7 @@
         </is>
       </c>
       <c r="I84" s="2" t="n">
-        <v>726</v>
+        <v>696</v>
       </c>
       <c r="J84" s="4" t="inlineStr">
         <is>
@@ -4829,7 +4829,7 @@
         </is>
       </c>
       <c r="I85" s="2" t="n">
-        <v>1665</v>
+        <v>793</v>
       </c>
       <c r="J85" s="4" t="inlineStr">
         <is>
@@ -4880,7 +4880,7 @@
         </is>
       </c>
       <c r="I86" s="2" t="n">
-        <v>680</v>
+        <v>713</v>
       </c>
       <c r="J86" s="4" t="inlineStr">
         <is>
@@ -4931,7 +4931,7 @@
         </is>
       </c>
       <c r="I87" s="2" t="n">
-        <v>2779</v>
+        <v>809</v>
       </c>
       <c r="J87" s="4" t="inlineStr">
         <is>
@@ -4982,7 +4982,7 @@
         </is>
       </c>
       <c r="I88" s="2" t="n">
-        <v>275</v>
+        <v>312</v>
       </c>
       <c r="J88" s="4" t="inlineStr">
         <is>
@@ -5033,7 +5033,7 @@
         </is>
       </c>
       <c r="I89" s="2" t="n">
-        <v>260</v>
+        <v>300</v>
       </c>
       <c r="J89" s="4" t="inlineStr">
         <is>
@@ -5084,7 +5084,7 @@
         </is>
       </c>
       <c r="I90" s="2" t="n">
-        <v>283</v>
+        <v>313</v>
       </c>
       <c r="J90" s="4" t="inlineStr">
         <is>
@@ -5135,7 +5135,7 @@
         </is>
       </c>
       <c r="I91" s="2" t="n">
-        <v>266</v>
+        <v>342</v>
       </c>
       <c r="J91" s="4" t="inlineStr">
         <is>
@@ -5186,7 +5186,7 @@
         </is>
       </c>
       <c r="I92" s="2" t="n">
-        <v>254</v>
+        <v>314</v>
       </c>
       <c r="J92" s="4" t="inlineStr">
         <is>
@@ -5237,7 +5237,7 @@
         </is>
       </c>
       <c r="I93" s="2" t="n">
-        <v>590</v>
+        <v>289</v>
       </c>
       <c r="J93" s="4" t="inlineStr">
         <is>
@@ -5288,7 +5288,7 @@
         </is>
       </c>
       <c r="I94" s="2" t="n">
-        <v>262</v>
+        <v>279</v>
       </c>
       <c r="J94" s="4" t="inlineStr">
         <is>
@@ -5339,7 +5339,7 @@
         </is>
       </c>
       <c r="I95" s="2" t="n">
-        <v>276</v>
+        <v>294</v>
       </c>
       <c r="J95" s="4" t="inlineStr">
         <is>
@@ -5390,7 +5390,7 @@
         </is>
       </c>
       <c r="I96" s="2" t="n">
-        <v>262</v>
+        <v>337</v>
       </c>
       <c r="J96" s="4" t="inlineStr">
         <is>
@@ -5441,7 +5441,7 @@
         </is>
       </c>
       <c r="I97" s="2" t="n">
-        <v>353</v>
+        <v>315</v>
       </c>
       <c r="J97" s="4" t="inlineStr">
         <is>
@@ -5492,7 +5492,7 @@
         </is>
       </c>
       <c r="I98" s="2" t="n">
-        <v>260</v>
+        <v>330</v>
       </c>
       <c r="J98" s="4" t="inlineStr">
         <is>
@@ -5543,7 +5543,7 @@
         </is>
       </c>
       <c r="I99" s="2" t="n">
-        <v>270</v>
+        <v>284</v>
       </c>
       <c r="J99" s="4" t="inlineStr">
         <is>
@@ -5594,7 +5594,7 @@
         </is>
       </c>
       <c r="I100" s="2" t="n">
-        <v>247</v>
+        <v>270</v>
       </c>
       <c r="J100" s="4" t="inlineStr">
         <is>
@@ -5645,7 +5645,7 @@
         </is>
       </c>
       <c r="I101" s="2" t="n">
-        <v>281</v>
+        <v>290</v>
       </c>
       <c r="J101" s="4" t="inlineStr">
         <is>
@@ -5696,7 +5696,7 @@
         </is>
       </c>
       <c r="I102" s="2" t="n">
-        <v>260</v>
+        <v>275</v>
       </c>
       <c r="J102" s="4" t="inlineStr">
         <is>
@@ -5747,7 +5747,7 @@
         </is>
       </c>
       <c r="I103" s="2" t="n">
-        <v>323</v>
+        <v>289</v>
       </c>
       <c r="J103" s="4" t="inlineStr">
         <is>
@@ -5798,7 +5798,7 @@
         </is>
       </c>
       <c r="I104" s="2" t="n">
-        <v>269</v>
+        <v>305</v>
       </c>
       <c r="J104" s="4" t="inlineStr">
         <is>
@@ -5849,7 +5849,7 @@
         </is>
       </c>
       <c r="I105" s="2" t="n">
-        <v>255</v>
+        <v>265</v>
       </c>
       <c r="J105" s="4" t="inlineStr">
         <is>
@@ -5900,7 +5900,7 @@
         </is>
       </c>
       <c r="I106" s="2" t="n">
-        <v>267</v>
+        <v>279</v>
       </c>
       <c r="J106" s="4" t="inlineStr">
         <is>
@@ -5951,7 +5951,7 @@
         </is>
       </c>
       <c r="I107" s="2" t="n">
-        <v>383</v>
+        <v>292</v>
       </c>
       <c r="J107" s="4" t="inlineStr">
         <is>
@@ -6002,7 +6002,7 @@
         </is>
       </c>
       <c r="I108" s="2" t="n">
-        <v>426</v>
+        <v>434</v>
       </c>
       <c r="J108" s="4" t="inlineStr">
         <is>
@@ -6053,7 +6053,7 @@
         </is>
       </c>
       <c r="I109" s="2" t="n">
-        <v>441</v>
+        <v>1902</v>
       </c>
       <c r="J109" s="4" t="inlineStr">
         <is>
@@ -6104,7 +6104,7 @@
         </is>
       </c>
       <c r="I110" s="2" t="n">
-        <v>425</v>
+        <v>470</v>
       </c>
       <c r="J110" s="4" t="inlineStr">
         <is>
@@ -6155,7 +6155,7 @@
         </is>
       </c>
       <c r="I111" s="2" t="n">
-        <v>438</v>
+        <v>397</v>
       </c>
       <c r="J111" s="4" t="inlineStr">
         <is>
@@ -6206,7 +6206,7 @@
         </is>
       </c>
       <c r="I112" s="2" t="n">
-        <v>472</v>
+        <v>514</v>
       </c>
       <c r="J112" s="4" t="inlineStr">
         <is>
@@ -6257,7 +6257,7 @@
         </is>
       </c>
       <c r="I113" s="2" t="n">
-        <v>571</v>
+        <v>510</v>
       </c>
       <c r="J113" s="4" t="inlineStr">
         <is>
@@ -6308,7 +6308,7 @@
         </is>
       </c>
       <c r="I114" s="2" t="n">
-        <v>1212</v>
+        <v>1152</v>
       </c>
       <c r="J114" s="4" t="inlineStr">
         <is>
@@ -6359,7 +6359,7 @@
         </is>
       </c>
       <c r="I115" s="2" t="n">
-        <v>428</v>
+        <v>939</v>
       </c>
       <c r="J115" s="4" t="inlineStr">
         <is>
@@ -6410,7 +6410,7 @@
         </is>
       </c>
       <c r="I116" s="2" t="n">
-        <v>403</v>
+        <v>398</v>
       </c>
       <c r="J116" s="4" t="inlineStr">
         <is>
@@ -6461,7 +6461,7 @@
         </is>
       </c>
       <c r="I117" s="2" t="n">
-        <v>428</v>
+        <v>397</v>
       </c>
       <c r="J117" s="4" t="inlineStr">
         <is>
@@ -6512,7 +6512,7 @@
         </is>
       </c>
       <c r="I118" s="2" t="n">
-        <v>457</v>
+        <v>513</v>
       </c>
       <c r="J118" s="4" t="inlineStr">
         <is>
@@ -6563,7 +6563,7 @@
         </is>
       </c>
       <c r="I119" s="2" t="n">
-        <v>482</v>
+        <v>406</v>
       </c>
       <c r="J119" s="4" t="inlineStr">
         <is>
@@ -6614,7 +6614,7 @@
         </is>
       </c>
       <c r="I120" s="2" t="n">
-        <v>514</v>
+        <v>449</v>
       </c>
       <c r="J120" s="4" t="inlineStr">
         <is>
@@ -6665,7 +6665,7 @@
         </is>
       </c>
       <c r="I121" s="2" t="n">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="J121" s="4" t="inlineStr">
         <is>
@@ -6716,7 +6716,7 @@
         </is>
       </c>
       <c r="I122" s="2" t="n">
-        <v>467</v>
+        <v>409</v>
       </c>
       <c r="J122" s="4" t="inlineStr">
         <is>
@@ -6767,7 +6767,7 @@
         </is>
       </c>
       <c r="I123" s="2" t="n">
-        <v>429</v>
+        <v>1225</v>
       </c>
       <c r="J123" s="4" t="inlineStr">
         <is>
@@ -6818,7 +6818,7 @@
         </is>
       </c>
       <c r="I124" s="2" t="n">
-        <v>445</v>
+        <v>420</v>
       </c>
       <c r="J124" s="4" t="inlineStr">
         <is>
@@ -6869,7 +6869,7 @@
         </is>
       </c>
       <c r="I125" s="2" t="n">
-        <v>620</v>
+        <v>409</v>
       </c>
       <c r="J125" s="4" t="inlineStr">
         <is>
@@ -6920,7 +6920,7 @@
         </is>
       </c>
       <c r="I126" s="2" t="n">
-        <v>454</v>
+        <v>414</v>
       </c>
       <c r="J126" s="4" t="inlineStr">
         <is>
@@ -6971,7 +6971,7 @@
         </is>
       </c>
       <c r="I127" s="2" t="n">
-        <v>424</v>
+        <v>434</v>
       </c>
       <c r="J127" s="4" t="inlineStr">
         <is>
@@ -7022,7 +7022,7 @@
         </is>
       </c>
       <c r="I128" s="2" t="n">
-        <v>3313</v>
+        <v>386</v>
       </c>
       <c r="J128" s="4" t="inlineStr">
         <is>
@@ -7073,7 +7073,7 @@
         </is>
       </c>
       <c r="I129" s="2" t="n">
-        <v>96</v>
+        <v>243</v>
       </c>
       <c r="J129" s="4" t="inlineStr">
         <is>
@@ -7124,7 +7124,7 @@
         </is>
       </c>
       <c r="I130" s="2" t="n">
-        <v>1119</v>
+        <v>966</v>
       </c>
       <c r="J130" s="4" t="inlineStr">
         <is>
@@ -7175,7 +7175,7 @@
         </is>
       </c>
       <c r="I131" s="2" t="n">
-        <v>611</v>
+        <v>322</v>
       </c>
       <c r="J131" s="4" t="inlineStr">
         <is>
@@ -7226,7 +7226,7 @@
         </is>
       </c>
       <c r="I132" s="2" t="n">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="J132" s="4" t="inlineStr">
         <is>
@@ -7277,7 +7277,7 @@
         </is>
       </c>
       <c r="I133" s="2" t="n">
-        <v>340</v>
+        <v>413</v>
       </c>
       <c r="J133" s="4" t="inlineStr">
         <is>
@@ -7328,7 +7328,7 @@
         </is>
       </c>
       <c r="I134" s="2" t="n">
-        <v>591</v>
+        <v>329</v>
       </c>
       <c r="J134" s="4" t="inlineStr">
         <is>
@@ -7379,7 +7379,7 @@
         </is>
       </c>
       <c r="I135" s="2" t="n">
-        <v>379</v>
+        <v>336</v>
       </c>
       <c r="J135" s="4" t="inlineStr">
         <is>
@@ -7430,7 +7430,7 @@
         </is>
       </c>
       <c r="I136" s="2" t="n">
-        <v>150</v>
+        <v>298</v>
       </c>
       <c r="J136" s="4" t="inlineStr">
         <is>
@@ -7481,7 +7481,7 @@
         </is>
       </c>
       <c r="I137" s="2" t="n">
-        <v>323</v>
+        <v>353</v>
       </c>
       <c r="J137" s="4" t="inlineStr">
         <is>
@@ -7532,7 +7532,7 @@
         </is>
       </c>
       <c r="I138" s="2" t="n">
-        <v>446</v>
+        <v>348</v>
       </c>
       <c r="J138" s="4" t="inlineStr">
         <is>
@@ -7583,7 +7583,7 @@
         </is>
       </c>
       <c r="I139" s="2" t="n">
-        <v>658</v>
+        <v>617</v>
       </c>
       <c r="J139" s="4" t="inlineStr">
         <is>
@@ -7634,7 +7634,7 @@
         </is>
       </c>
       <c r="I140" s="2" t="n">
-        <v>162</v>
+        <v>293</v>
       </c>
       <c r="J140" s="4" t="inlineStr">
         <is>
@@ -7685,7 +7685,7 @@
         </is>
       </c>
       <c r="I141" s="2" t="n">
-        <v>111</v>
+        <v>231</v>
       </c>
       <c r="J141" s="4" t="inlineStr">
         <is>
@@ -7736,7 +7736,7 @@
         </is>
       </c>
       <c r="I142" s="2" t="n">
-        <v>101</v>
+        <v>295</v>
       </c>
       <c r="J142" s="4" t="inlineStr">
         <is>
@@ -7787,7 +7787,7 @@
         </is>
       </c>
       <c r="I143" s="2" t="n">
-        <v>1236</v>
+        <v>1273</v>
       </c>
       <c r="J143" s="4" t="inlineStr">
         <is>
@@ -7838,7 +7838,7 @@
         </is>
       </c>
       <c r="I144" s="2" t="n">
-        <v>663</v>
+        <v>300</v>
       </c>
       <c r="J144" s="4" t="inlineStr">
         <is>
@@ -7889,7 +7889,7 @@
         </is>
       </c>
       <c r="I145" s="2" t="n">
-        <v>437</v>
+        <v>339</v>
       </c>
       <c r="J145" s="4" t="inlineStr">
         <is>
@@ -7940,7 +7940,7 @@
         </is>
       </c>
       <c r="I146" s="2" t="n">
-        <v>975</v>
+        <v>1117</v>
       </c>
       <c r="J146" s="4" t="inlineStr">
         <is>
@@ -7991,7 +7991,7 @@
         </is>
       </c>
       <c r="I147" s="2" t="n">
-        <v>322</v>
+        <v>390</v>
       </c>
       <c r="J147" s="4" t="inlineStr">
         <is>
@@ -8042,7 +8042,7 @@
         </is>
       </c>
       <c r="I148" s="2" t="n">
-        <v>266</v>
+        <v>277</v>
       </c>
       <c r="J148" s="4" t="inlineStr">
         <is>
@@ -8093,7 +8093,7 @@
         </is>
       </c>
       <c r="I149" s="2" t="n">
-        <v>59</v>
+        <v>382</v>
       </c>
       <c r="J149" s="4" t="inlineStr">
         <is>
@@ -8144,7 +8144,7 @@
         </is>
       </c>
       <c r="I150" s="2" t="n">
-        <v>985</v>
+        <v>583</v>
       </c>
       <c r="J150" s="4" t="inlineStr">
         <is>
@@ -8195,7 +8195,7 @@
         </is>
       </c>
       <c r="I151" s="2" t="n">
-        <v>302</v>
+        <v>278</v>
       </c>
       <c r="J151" s="4" t="inlineStr">
         <is>
@@ -8246,7 +8246,7 @@
         </is>
       </c>
       <c r="I152" s="2" t="n">
-        <v>112</v>
+        <v>306</v>
       </c>
       <c r="J152" s="4" t="inlineStr">
         <is>
@@ -8297,7 +8297,7 @@
         </is>
       </c>
       <c r="I153" s="2" t="n">
-        <v>536</v>
+        <v>319</v>
       </c>
       <c r="J153" s="4" t="inlineStr">
         <is>
@@ -8348,7 +8348,7 @@
         </is>
       </c>
       <c r="I154" s="2" t="n">
-        <v>317</v>
+        <v>325</v>
       </c>
       <c r="J154" s="4" t="inlineStr">
         <is>
@@ -8399,7 +8399,7 @@
         </is>
       </c>
       <c r="I155" s="2" t="n">
-        <v>276</v>
+        <v>355</v>
       </c>
       <c r="J155" s="4" t="inlineStr">
         <is>
@@ -8450,7 +8450,7 @@
         </is>
       </c>
       <c r="I156" s="2" t="n">
-        <v>88</v>
+        <v>260</v>
       </c>
       <c r="J156" s="4" t="inlineStr">
         <is>
@@ -8501,7 +8501,7 @@
         </is>
       </c>
       <c r="I157" s="2" t="n">
-        <v>302</v>
+        <v>285</v>
       </c>
       <c r="J157" s="4" t="inlineStr">
         <is>
@@ -8552,7 +8552,7 @@
         </is>
       </c>
       <c r="I158" s="2" t="n">
-        <v>537</v>
+        <v>295</v>
       </c>
       <c r="J158" s="4" t="inlineStr">
         <is>
@@ -8603,7 +8603,7 @@
         </is>
       </c>
       <c r="I159" s="2" t="n">
-        <v>429</v>
+        <v>468</v>
       </c>
       <c r="J159" s="4" t="inlineStr">
         <is>
@@ -8654,7 +8654,7 @@
         </is>
       </c>
       <c r="I160" s="2" t="n">
-        <v>66</v>
+        <v>219</v>
       </c>
       <c r="J160" s="4" t="inlineStr">
         <is>
@@ -8705,7 +8705,7 @@
         </is>
       </c>
       <c r="I161" s="2" t="n">
-        <v>73</v>
+        <v>265</v>
       </c>
       <c r="J161" s="4" t="inlineStr">
         <is>
@@ -8756,7 +8756,7 @@
         </is>
       </c>
       <c r="I162" s="2" t="n">
-        <v>63</v>
+        <v>268</v>
       </c>
       <c r="J162" s="4" t="inlineStr">
         <is>
@@ -8807,7 +8807,7 @@
         </is>
       </c>
       <c r="I163" s="2" t="n">
-        <v>729</v>
+        <v>1077</v>
       </c>
       <c r="J163" s="4" t="inlineStr">
         <is>
@@ -8858,7 +8858,7 @@
         </is>
       </c>
       <c r="I164" s="2" t="n">
-        <v>265</v>
+        <v>290</v>
       </c>
       <c r="J164" s="4" t="inlineStr">
         <is>
@@ -8909,7 +8909,7 @@
         </is>
       </c>
       <c r="I165" s="2" t="n">
-        <v>347</v>
+        <v>295</v>
       </c>
       <c r="J165" s="4" t="inlineStr">
         <is>
@@ -8960,7 +8960,7 @@
         </is>
       </c>
       <c r="I166" s="2" t="n">
-        <v>738</v>
+        <v>751</v>
       </c>
       <c r="J166" s="4" t="inlineStr">
         <is>
@@ -9011,7 +9011,7 @@
         </is>
       </c>
       <c r="I167" s="2" t="n">
-        <v>694</v>
+        <v>302</v>
       </c>
       <c r="J167" s="4" t="inlineStr">
         <is>
@@ -9062,7 +9062,7 @@
         </is>
       </c>
       <c r="I168" s="2" t="n">
-        <v>743</v>
+        <v>659</v>
       </c>
       <c r="J168" s="4" t="inlineStr">
         <is>
@@ -9113,7 +9113,7 @@
         </is>
       </c>
       <c r="I169" s="2" t="n">
-        <v>866</v>
+        <v>658</v>
       </c>
       <c r="J169" s="4" t="inlineStr">
         <is>
@@ -9164,7 +9164,7 @@
         </is>
       </c>
       <c r="I170" s="2" t="n">
-        <v>653</v>
+        <v>721</v>
       </c>
       <c r="J170" s="4" t="inlineStr">
         <is>
@@ -9215,7 +9215,7 @@
         </is>
       </c>
       <c r="I171" s="2" t="n">
-        <v>686</v>
+        <v>692</v>
       </c>
       <c r="J171" s="4" t="inlineStr">
         <is>
@@ -9266,7 +9266,7 @@
         </is>
       </c>
       <c r="I172" s="2" t="n">
-        <v>620</v>
+        <v>765</v>
       </c>
       <c r="J172" s="4" t="inlineStr">
         <is>
@@ -9317,7 +9317,7 @@
         </is>
       </c>
       <c r="I173" s="2" t="n">
-        <v>650</v>
+        <v>704</v>
       </c>
       <c r="J173" s="4" t="inlineStr">
         <is>
@@ -9368,7 +9368,7 @@
         </is>
       </c>
       <c r="I174" s="2" t="n">
-        <v>605</v>
+        <v>669</v>
       </c>
       <c r="J174" s="4" t="inlineStr">
         <is>
@@ -9419,7 +9419,7 @@
         </is>
       </c>
       <c r="I175" s="2" t="n">
-        <v>1025</v>
+        <v>685</v>
       </c>
       <c r="J175" s="4" t="inlineStr">
         <is>
@@ -9470,7 +9470,7 @@
         </is>
       </c>
       <c r="I176" s="2" t="n">
-        <v>648</v>
+        <v>658</v>
       </c>
       <c r="J176" s="4" t="inlineStr">
         <is>
@@ -9521,7 +9521,7 @@
         </is>
       </c>
       <c r="I177" s="2" t="n">
-        <v>897</v>
+        <v>646</v>
       </c>
       <c r="J177" s="4" t="inlineStr">
         <is>
@@ -9572,7 +9572,7 @@
         </is>
       </c>
       <c r="I178" s="2" t="n">
-        <v>710</v>
+        <v>641</v>
       </c>
       <c r="J178" s="4" t="inlineStr">
         <is>
@@ -9623,7 +9623,7 @@
         </is>
       </c>
       <c r="I179" s="2" t="n">
-        <v>765</v>
+        <v>769</v>
       </c>
       <c r="J179" s="4" t="inlineStr">
         <is>
@@ -9674,7 +9674,7 @@
         </is>
       </c>
       <c r="I180" s="2" t="n">
-        <v>692</v>
+        <v>731</v>
       </c>
       <c r="J180" s="4" t="inlineStr">
         <is>
@@ -9725,7 +9725,7 @@
         </is>
       </c>
       <c r="I181" s="2" t="n">
-        <v>665</v>
+        <v>678</v>
       </c>
       <c r="J181" s="4" t="inlineStr">
         <is>
@@ -9776,7 +9776,7 @@
         </is>
       </c>
       <c r="I182" s="2" t="n">
-        <v>690</v>
+        <v>695</v>
       </c>
       <c r="J182" s="4" t="inlineStr">
         <is>
@@ -9827,7 +9827,7 @@
         </is>
       </c>
       <c r="I183" s="2" t="n">
-        <v>628</v>
+        <v>661</v>
       </c>
       <c r="J183" s="4" t="inlineStr">
         <is>
@@ -9878,7 +9878,7 @@
         </is>
       </c>
       <c r="I184" s="2" t="n">
-        <v>861</v>
+        <v>639</v>
       </c>
       <c r="J184" s="4" t="inlineStr">
         <is>
@@ -9929,7 +9929,7 @@
         </is>
       </c>
       <c r="I185" s="2" t="n">
-        <v>639</v>
+        <v>684</v>
       </c>
       <c r="J185" s="4" t="inlineStr">
         <is>
@@ -9980,7 +9980,7 @@
         </is>
       </c>
       <c r="I186" s="2" t="n">
-        <v>638</v>
+        <v>654</v>
       </c>
       <c r="J186" s="4" t="inlineStr">
         <is>
@@ -10031,7 +10031,7 @@
         </is>
       </c>
       <c r="I187" s="2" t="n">
-        <v>647</v>
+        <v>681</v>
       </c>
       <c r="J187" s="4" t="inlineStr">
         <is>
@@ -10082,7 +10082,7 @@
         </is>
       </c>
       <c r="I188" s="2" t="n">
-        <v>817</v>
+        <v>804</v>
       </c>
       <c r="J188" s="4" t="inlineStr">
         <is>
@@ -10133,7 +10133,7 @@
         </is>
       </c>
       <c r="I189" s="2" t="n">
-        <v>826</v>
+        <v>717</v>
       </c>
       <c r="J189" s="4" t="inlineStr">
         <is>
@@ -10184,7 +10184,7 @@
         </is>
       </c>
       <c r="I190" s="2" t="n">
-        <v>835</v>
+        <v>740</v>
       </c>
       <c r="J190" s="4" t="inlineStr">
         <is>
@@ -10235,7 +10235,7 @@
         </is>
       </c>
       <c r="I191" s="2" t="n">
-        <v>850</v>
+        <v>741</v>
       </c>
       <c r="J191" s="4" t="inlineStr">
         <is>
@@ -10286,7 +10286,7 @@
         </is>
       </c>
       <c r="I192" s="2" t="n">
-        <v>778</v>
+        <v>884</v>
       </c>
       <c r="J192" s="4" t="inlineStr">
         <is>
@@ -10337,7 +10337,7 @@
         </is>
       </c>
       <c r="I193" s="2" t="n">
-        <v>859</v>
+        <v>811</v>
       </c>
       <c r="J193" s="4" t="inlineStr">
         <is>
@@ -10388,7 +10388,7 @@
         </is>
       </c>
       <c r="I194" s="2" t="n">
-        <v>837</v>
+        <v>787</v>
       </c>
       <c r="J194" s="4" t="inlineStr">
         <is>
@@ -10439,7 +10439,7 @@
         </is>
       </c>
       <c r="I195" s="2" t="n">
-        <v>718</v>
+        <v>889</v>
       </c>
       <c r="J195" s="4" t="inlineStr">
         <is>
@@ -10490,7 +10490,7 @@
         </is>
       </c>
       <c r="I196" s="2" t="n">
-        <v>756</v>
+        <v>780</v>
       </c>
       <c r="J196" s="4" t="inlineStr">
         <is>
@@ -10541,7 +10541,7 @@
         </is>
       </c>
       <c r="I197" s="2" t="n">
-        <v>807</v>
+        <v>775</v>
       </c>
       <c r="J197" s="4" t="inlineStr">
         <is>
@@ -10592,7 +10592,7 @@
         </is>
       </c>
       <c r="I198" s="2" t="n">
-        <v>782</v>
+        <v>790</v>
       </c>
       <c r="J198" s="4" t="inlineStr">
         <is>
@@ -10643,7 +10643,7 @@
         </is>
       </c>
       <c r="I199" s="2" t="n">
-        <v>870</v>
+        <v>771</v>
       </c>
       <c r="J199" s="4" t="inlineStr">
         <is>
@@ -10694,7 +10694,7 @@
         </is>
       </c>
       <c r="I200" s="2" t="n">
-        <v>905</v>
+        <v>759</v>
       </c>
       <c r="J200" s="4" t="inlineStr">
         <is>
@@ -10745,7 +10745,7 @@
         </is>
       </c>
       <c r="I201" s="2" t="n">
-        <v>737</v>
+        <v>860</v>
       </c>
       <c r="J201" s="4" t="inlineStr">
         <is>
@@ -10796,7 +10796,7 @@
         </is>
       </c>
       <c r="I202" s="2" t="n">
-        <v>703</v>
+        <v>794</v>
       </c>
       <c r="J202" s="4" t="inlineStr">
         <is>
@@ -10847,7 +10847,7 @@
         </is>
       </c>
       <c r="I203" s="2" t="n">
-        <v>848</v>
+        <v>786</v>
       </c>
       <c r="J203" s="4" t="inlineStr">
         <is>
@@ -10898,7 +10898,7 @@
         </is>
       </c>
       <c r="I204" s="2" t="n">
-        <v>1071</v>
+        <v>923</v>
       </c>
       <c r="J204" s="4" t="inlineStr">
         <is>
@@ -10949,7 +10949,7 @@
         </is>
       </c>
       <c r="I205" s="2" t="n">
-        <v>729</v>
+        <v>791</v>
       </c>
       <c r="J205" s="4" t="inlineStr">
         <is>
@@ -11000,7 +11000,7 @@
         </is>
       </c>
       <c r="I206" s="2" t="n">
-        <v>809</v>
+        <v>720</v>
       </c>
       <c r="J206" s="4" t="inlineStr">
         <is>
@@ -11051,7 +11051,7 @@
         </is>
       </c>
       <c r="I207" s="2" t="n">
-        <v>850</v>
+        <v>778</v>
       </c>
       <c r="J207" s="4" t="inlineStr">
         <is>
@@ -11102,7 +11102,7 @@
         </is>
       </c>
       <c r="I208" s="2" t="n">
-        <v>865</v>
+        <v>794</v>
       </c>
       <c r="J208" s="4" t="inlineStr">
         <is>
@@ -11153,7 +11153,7 @@
         </is>
       </c>
       <c r="I209" s="2" t="n">
-        <v>788</v>
+        <v>844</v>
       </c>
       <c r="J209" s="4" t="inlineStr">
         <is>
@@ -11204,7 +11204,7 @@
         </is>
       </c>
       <c r="I210" s="2" t="n">
-        <v>842</v>
+        <v>773</v>
       </c>
       <c r="J210" s="4" t="inlineStr">
         <is>
@@ -11255,7 +11255,7 @@
         </is>
       </c>
       <c r="I211" s="2" t="n">
-        <v>773</v>
+        <v>742</v>
       </c>
       <c r="J211" s="4" t="inlineStr">
         <is>
@@ -11306,7 +11306,7 @@
         </is>
       </c>
       <c r="I212" s="2" t="n">
-        <v>795</v>
+        <v>765</v>
       </c>
       <c r="J212" s="4" t="inlineStr">
         <is>
@@ -11357,7 +11357,7 @@
         </is>
       </c>
       <c r="I213" s="2" t="n">
-        <v>741</v>
+        <v>737</v>
       </c>
       <c r="J213" s="4" t="inlineStr">
         <is>
@@ -11408,7 +11408,7 @@
         </is>
       </c>
       <c r="I214" s="2" t="n">
-        <v>710</v>
+        <v>803</v>
       </c>
       <c r="J214" s="4" t="inlineStr">
         <is>
@@ -11459,7 +11459,7 @@
         </is>
       </c>
       <c r="I215" s="2" t="n">
-        <v>743</v>
+        <v>761</v>
       </c>
       <c r="J215" s="4" t="inlineStr">
         <is>
@@ -11510,7 +11510,7 @@
         </is>
       </c>
       <c r="I216" s="2" t="n">
-        <v>782</v>
+        <v>749</v>
       </c>
       <c r="J216" s="4" t="inlineStr">
         <is>
@@ -11561,7 +11561,7 @@
         </is>
       </c>
       <c r="I217" s="2" t="n">
-        <v>867</v>
+        <v>724</v>
       </c>
       <c r="J217" s="4" t="inlineStr">
         <is>
@@ -11612,7 +11612,7 @@
         </is>
       </c>
       <c r="I218" s="2" t="n">
-        <v>1834</v>
+        <v>846</v>
       </c>
       <c r="J218" s="4" t="inlineStr">
         <is>
@@ -11663,7 +11663,7 @@
         </is>
       </c>
       <c r="I219" s="2" t="n">
-        <v>831</v>
+        <v>842</v>
       </c>
       <c r="J219" s="4" t="inlineStr">
         <is>
@@ -11714,7 +11714,7 @@
         </is>
       </c>
       <c r="I220" s="2" t="n">
-        <v>764</v>
+        <v>731</v>
       </c>
       <c r="J220" s="4" t="inlineStr">
         <is>
@@ -11765,7 +11765,7 @@
         </is>
       </c>
       <c r="I221" s="2" t="n">
-        <v>735</v>
+        <v>772</v>
       </c>
       <c r="J221" s="4" t="inlineStr">
         <is>
@@ -11816,7 +11816,7 @@
         </is>
       </c>
       <c r="I222" s="2" t="n">
-        <v>914</v>
+        <v>774</v>
       </c>
       <c r="J222" s="4" t="inlineStr">
         <is>
@@ -11867,7 +11867,7 @@
         </is>
       </c>
       <c r="I223" s="2" t="n">
-        <v>972</v>
+        <v>849</v>
       </c>
       <c r="J223" s="4" t="inlineStr">
         <is>
@@ -11918,7 +11918,7 @@
         </is>
       </c>
       <c r="I224" s="2" t="n">
-        <v>738</v>
+        <v>841</v>
       </c>
       <c r="J224" s="4" t="inlineStr">
         <is>
@@ -11969,7 +11969,7 @@
         </is>
       </c>
       <c r="I225" s="2" t="n">
-        <v>822</v>
+        <v>799</v>
       </c>
       <c r="J225" s="4" t="inlineStr">
         <is>
@@ -12020,7 +12020,7 @@
         </is>
       </c>
       <c r="I226" s="2" t="n">
-        <v>750</v>
+        <v>840</v>
       </c>
       <c r="J226" s="4" t="inlineStr">
         <is>
@@ -12071,7 +12071,7 @@
         </is>
       </c>
       <c r="I227" s="2" t="n">
-        <v>764</v>
+        <v>795</v>
       </c>
       <c r="J227" s="4" t="inlineStr">
         <is>
@@ -12122,7 +12122,7 @@
         </is>
       </c>
       <c r="I228" s="2" t="n">
-        <v>317</v>
+        <v>289</v>
       </c>
       <c r="J228" s="4" t="inlineStr">
         <is>
@@ -12173,7 +12173,7 @@
         </is>
       </c>
       <c r="I229" s="2" t="n">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="J229" s="4" t="inlineStr">
         <is>
@@ -12224,7 +12224,7 @@
         </is>
       </c>
       <c r="I230" s="2" t="n">
-        <v>404</v>
+        <v>416</v>
       </c>
       <c r="J230" s="4" t="inlineStr">
         <is>
@@ -12275,7 +12275,7 @@
         </is>
       </c>
       <c r="I231" s="2" t="n">
-        <v>330</v>
+        <v>287</v>
       </c>
       <c r="J231" s="4" t="inlineStr">
         <is>
@@ -12326,7 +12326,7 @@
         </is>
       </c>
       <c r="I232" s="2" t="n">
-        <v>336</v>
+        <v>319</v>
       </c>
       <c r="J232" s="4" t="inlineStr">
         <is>
@@ -12377,7 +12377,7 @@
         </is>
       </c>
       <c r="I233" s="2" t="n">
-        <v>323</v>
+        <v>630</v>
       </c>
       <c r="J233" s="4" t="inlineStr">
         <is>
@@ -12428,7 +12428,7 @@
         </is>
       </c>
       <c r="I234" s="2" t="n">
-        <v>287</v>
+        <v>389</v>
       </c>
       <c r="J234" s="4" t="inlineStr">
         <is>
@@ -12479,7 +12479,7 @@
         </is>
       </c>
       <c r="I235" s="2" t="n">
-        <v>315</v>
+        <v>295</v>
       </c>
       <c r="J235" s="4" t="inlineStr">
         <is>
@@ -12530,7 +12530,7 @@
         </is>
       </c>
       <c r="I236" s="2" t="n">
-        <v>270</v>
+        <v>312</v>
       </c>
       <c r="J236" s="4" t="inlineStr">
         <is>
@@ -12581,7 +12581,7 @@
         </is>
       </c>
       <c r="I237" s="2" t="n">
-        <v>272</v>
+        <v>303</v>
       </c>
       <c r="J237" s="4" t="inlineStr">
         <is>
@@ -12632,7 +12632,7 @@
         </is>
       </c>
       <c r="I238" s="2" t="n">
-        <v>301</v>
+        <v>289</v>
       </c>
       <c r="J238" s="4" t="inlineStr">
         <is>
@@ -12683,7 +12683,7 @@
         </is>
       </c>
       <c r="I239" s="2" t="n">
-        <v>360</v>
+        <v>299</v>
       </c>
       <c r="J239" s="4" t="inlineStr">
         <is>
@@ -12734,7 +12734,7 @@
         </is>
       </c>
       <c r="I240" s="2" t="n">
-        <v>428</v>
+        <v>277</v>
       </c>
       <c r="J240" s="4" t="inlineStr">
         <is>
@@ -12785,7 +12785,7 @@
         </is>
       </c>
       <c r="I241" s="2" t="n">
-        <v>341</v>
+        <v>300</v>
       </c>
       <c r="J241" s="4" t="inlineStr">
         <is>
@@ -12836,7 +12836,7 @@
         </is>
       </c>
       <c r="I242" s="2" t="n">
-        <v>474</v>
+        <v>283</v>
       </c>
       <c r="J242" s="4" t="inlineStr">
         <is>
@@ -12887,7 +12887,7 @@
         </is>
       </c>
       <c r="I243" s="2" t="n">
-        <v>298</v>
+        <v>277</v>
       </c>
       <c r="J243" s="4" t="inlineStr">
         <is>
@@ -12938,7 +12938,7 @@
         </is>
       </c>
       <c r="I244" s="2" t="n">
-        <v>283</v>
+        <v>294</v>
       </c>
       <c r="J244" s="4" t="inlineStr">
         <is>
@@ -12989,7 +12989,7 @@
         </is>
       </c>
       <c r="I245" s="2" t="n">
-        <v>323</v>
+        <v>352</v>
       </c>
       <c r="J245" s="4" t="inlineStr">
         <is>
@@ -13040,7 +13040,7 @@
         </is>
       </c>
       <c r="I246" s="2" t="n">
-        <v>289</v>
+        <v>271</v>
       </c>
       <c r="J246" s="4" t="inlineStr">
         <is>
@@ -13091,7 +13091,7 @@
         </is>
       </c>
       <c r="I247" s="2" t="n">
-        <v>290</v>
+        <v>310</v>
       </c>
       <c r="J247" s="4" t="inlineStr">
         <is>
@@ -13142,7 +13142,7 @@
         </is>
       </c>
       <c r="I248" s="2" t="n">
-        <v>470</v>
+        <v>451</v>
       </c>
       <c r="J248" s="4" t="inlineStr">
         <is>
@@ -13193,7 +13193,7 @@
         </is>
       </c>
       <c r="I249" s="2" t="n">
-        <v>423</v>
+        <v>1049</v>
       </c>
       <c r="J249" s="4" t="inlineStr">
         <is>
@@ -13244,7 +13244,7 @@
         </is>
       </c>
       <c r="I250" s="2" t="n">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="J250" s="4" t="inlineStr">
         <is>
@@ -13295,7 +13295,7 @@
         </is>
       </c>
       <c r="I251" s="2" t="n">
-        <v>399</v>
+        <v>416</v>
       </c>
       <c r="J251" s="4" t="inlineStr">
         <is>
@@ -13346,7 +13346,7 @@
         </is>
       </c>
       <c r="I252" s="2" t="n">
-        <v>499</v>
+        <v>550</v>
       </c>
       <c r="J252" s="4" t="inlineStr">
         <is>
@@ -13397,7 +13397,7 @@
         </is>
       </c>
       <c r="I253" s="2" t="n">
-        <v>436</v>
+        <v>568</v>
       </c>
       <c r="J253" s="4" t="inlineStr">
         <is>
@@ -13448,7 +13448,7 @@
         </is>
       </c>
       <c r="I254" s="2" t="n">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="J254" s="4" t="inlineStr">
         <is>
@@ -13499,7 +13499,7 @@
         </is>
       </c>
       <c r="I255" s="2" t="n">
-        <v>477</v>
+        <v>456</v>
       </c>
       <c r="J255" s="4" t="inlineStr">
         <is>
@@ -13550,7 +13550,7 @@
         </is>
       </c>
       <c r="I256" s="2" t="n">
-        <v>484</v>
+        <v>435</v>
       </c>
       <c r="J256" s="4" t="inlineStr">
         <is>
@@ -13601,7 +13601,7 @@
         </is>
       </c>
       <c r="I257" s="2" t="n">
-        <v>566</v>
+        <v>589</v>
       </c>
       <c r="J257" s="4" t="inlineStr">
         <is>
@@ -13652,7 +13652,7 @@
         </is>
       </c>
       <c r="I258" s="2" t="n">
-        <v>516</v>
+        <v>447</v>
       </c>
       <c r="J258" s="4" t="inlineStr">
         <is>
@@ -13703,7 +13703,7 @@
         </is>
       </c>
       <c r="I259" s="2" t="n">
-        <v>492</v>
+        <v>387</v>
       </c>
       <c r="J259" s="4" t="inlineStr">
         <is>
@@ -13754,7 +13754,7 @@
         </is>
       </c>
       <c r="I260" s="2" t="n">
-        <v>419</v>
+        <v>427</v>
       </c>
       <c r="J260" s="4" t="inlineStr">
         <is>
@@ -13805,7 +13805,7 @@
         </is>
       </c>
       <c r="I261" s="2" t="n">
-        <v>502</v>
+        <v>428</v>
       </c>
       <c r="J261" s="4" t="inlineStr">
         <is>
@@ -13856,7 +13856,7 @@
         </is>
       </c>
       <c r="I262" s="2" t="n">
-        <v>565</v>
+        <v>910</v>
       </c>
       <c r="J262" s="4" t="inlineStr">
         <is>
@@ -13907,7 +13907,7 @@
         </is>
       </c>
       <c r="I263" s="2" t="n">
-        <v>530</v>
+        <v>418</v>
       </c>
       <c r="J263" s="4" t="inlineStr">
         <is>
@@ -13958,7 +13958,7 @@
         </is>
       </c>
       <c r="I264" s="2" t="n">
-        <v>558</v>
+        <v>442</v>
       </c>
       <c r="J264" s="4" t="inlineStr">
         <is>
@@ -14009,7 +14009,7 @@
         </is>
       </c>
       <c r="I265" s="2" t="n">
-        <v>542</v>
+        <v>1015</v>
       </c>
       <c r="J265" s="4" t="inlineStr">
         <is>
@@ -14060,7 +14060,7 @@
         </is>
       </c>
       <c r="I266" s="2" t="n">
-        <v>418</v>
+        <v>463</v>
       </c>
       <c r="J266" s="4" t="inlineStr">
         <is>
@@ -14111,7 +14111,7 @@
         </is>
       </c>
       <c r="I267" s="2" t="n">
-        <v>790</v>
+        <v>398</v>
       </c>
       <c r="J267" s="4" t="inlineStr">
         <is>
@@ -14162,7 +14162,7 @@
         </is>
       </c>
       <c r="I268" s="2" t="n">
-        <v>426</v>
+        <v>444</v>
       </c>
       <c r="J268" s="4" t="inlineStr">
         <is>
@@ -14213,7 +14213,7 @@
         </is>
       </c>
       <c r="I269" s="2" t="n">
-        <v>421</v>
+        <v>407</v>
       </c>
       <c r="J269" s="4" t="inlineStr">
         <is>
@@ -14264,7 +14264,7 @@
         </is>
       </c>
       <c r="I270" s="2" t="n">
-        <v>420</v>
+        <v>481</v>
       </c>
       <c r="J270" s="4" t="inlineStr">
         <is>
@@ -14315,7 +14315,7 @@
         </is>
       </c>
       <c r="I271" s="2" t="n">
-        <v>1528</v>
+        <v>440</v>
       </c>
       <c r="J271" s="4" t="inlineStr">
         <is>
@@ -14366,7 +14366,7 @@
         </is>
       </c>
       <c r="I272" s="2" t="n">
-        <v>464</v>
+        <v>452</v>
       </c>
       <c r="J272" s="4" t="inlineStr">
         <is>
@@ -14417,7 +14417,7 @@
         </is>
       </c>
       <c r="I273" s="2" t="n">
-        <v>511</v>
+        <v>458</v>
       </c>
       <c r="J273" s="4" t="inlineStr">
         <is>
@@ -14468,7 +14468,7 @@
         </is>
       </c>
       <c r="I274" s="2" t="n">
-        <v>883</v>
+        <v>416</v>
       </c>
       <c r="J274" s="4" t="inlineStr">
         <is>
@@ -14519,7 +14519,7 @@
         </is>
       </c>
       <c r="I275" s="2" t="n">
-        <v>465</v>
+        <v>435</v>
       </c>
       <c r="J275" s="4" t="inlineStr">
         <is>
@@ -14570,7 +14570,7 @@
         </is>
       </c>
       <c r="I276" s="2" t="n">
-        <v>1524</v>
+        <v>446</v>
       </c>
       <c r="J276" s="4" t="inlineStr">
         <is>
@@ -14621,7 +14621,7 @@
         </is>
       </c>
       <c r="I277" s="2" t="n">
-        <v>480</v>
+        <v>1463</v>
       </c>
       <c r="J277" s="4" t="inlineStr">
         <is>
@@ -14672,7 +14672,7 @@
         </is>
       </c>
       <c r="I278" s="2" t="n">
-        <v>477</v>
+        <v>453</v>
       </c>
       <c r="J278" s="4" t="inlineStr">
         <is>
@@ -14723,7 +14723,7 @@
         </is>
       </c>
       <c r="I279" s="2" t="n">
-        <v>526</v>
+        <v>452</v>
       </c>
       <c r="J279" s="4" t="inlineStr">
         <is>
@@ -14774,7 +14774,7 @@
         </is>
       </c>
       <c r="I280" s="2" t="n">
-        <v>426</v>
+        <v>438</v>
       </c>
       <c r="J280" s="4" t="inlineStr">
         <is>
@@ -14825,7 +14825,7 @@
         </is>
       </c>
       <c r="I281" s="2" t="n">
-        <v>484</v>
+        <v>469</v>
       </c>
       <c r="J281" s="4" t="inlineStr">
         <is>
@@ -14927,7 +14927,7 @@
         </is>
       </c>
       <c r="I283" s="2" t="n">
-        <v>1441</v>
+        <v>416</v>
       </c>
       <c r="J283" s="4" t="inlineStr">
         <is>
@@ -14978,7 +14978,7 @@
         </is>
       </c>
       <c r="I284" s="2" t="n">
-        <v>428</v>
+        <v>457</v>
       </c>
       <c r="J284" s="4" t="inlineStr">
         <is>
@@ -15029,7 +15029,7 @@
         </is>
       </c>
       <c r="I285" s="2" t="n">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="J285" s="4" t="inlineStr">
         <is>
@@ -15080,7 +15080,7 @@
         </is>
       </c>
       <c r="I286" s="2" t="n">
-        <v>438</v>
+        <v>1438</v>
       </c>
       <c r="J286" s="4" t="inlineStr">
         <is>
@@ -15131,7 +15131,7 @@
         </is>
       </c>
       <c r="I287" s="2" t="n">
-        <v>446</v>
+        <v>430</v>
       </c>
       <c r="J287" s="4" t="inlineStr">
         <is>
@@ -15182,7 +15182,7 @@
         </is>
       </c>
       <c r="I288" s="2" t="n">
-        <v>749</v>
+        <v>1157</v>
       </c>
       <c r="J288" s="4" t="inlineStr">
         <is>
@@ -15233,7 +15233,7 @@
         </is>
       </c>
       <c r="I289" s="2" t="n">
-        <v>433</v>
+        <v>472</v>
       </c>
       <c r="J289" s="4" t="inlineStr">
         <is>
@@ -15284,7 +15284,7 @@
         </is>
       </c>
       <c r="I290" s="2" t="n">
-        <v>417</v>
+        <v>445</v>
       </c>
       <c r="J290" s="4" t="inlineStr">
         <is>
@@ -15335,7 +15335,7 @@
         </is>
       </c>
       <c r="I291" s="2" t="n">
-        <v>462</v>
+        <v>433</v>
       </c>
       <c r="J291" s="4" t="inlineStr">
         <is>
@@ -15386,7 +15386,7 @@
         </is>
       </c>
       <c r="I292" s="2" t="n">
-        <v>599</v>
+        <v>516</v>
       </c>
       <c r="J292" s="4" t="inlineStr">
         <is>
@@ -15437,7 +15437,7 @@
         </is>
       </c>
       <c r="I293" s="2" t="n">
-        <v>522</v>
+        <v>546</v>
       </c>
       <c r="J293" s="4" t="inlineStr">
         <is>
@@ -15488,7 +15488,7 @@
         </is>
       </c>
       <c r="I294" s="2" t="n">
-        <v>524</v>
+        <v>433</v>
       </c>
       <c r="J294" s="4" t="inlineStr">
         <is>
@@ -15539,7 +15539,7 @@
         </is>
       </c>
       <c r="I295" s="2" t="n">
-        <v>492</v>
+        <v>433</v>
       </c>
       <c r="J295" s="4" t="inlineStr">
         <is>
@@ -15590,7 +15590,7 @@
         </is>
       </c>
       <c r="I296" s="2" t="n">
-        <v>424</v>
+        <v>443</v>
       </c>
       <c r="J296" s="4" t="inlineStr">
         <is>
@@ -15641,7 +15641,7 @@
         </is>
       </c>
       <c r="I297" s="2" t="n">
-        <v>473</v>
+        <v>405</v>
       </c>
       <c r="J297" s="4" t="inlineStr">
         <is>
@@ -15692,7 +15692,7 @@
         </is>
       </c>
       <c r="I298" s="2" t="n">
-        <v>1296</v>
+        <v>432</v>
       </c>
       <c r="J298" s="4" t="inlineStr">
         <is>
@@ -15743,7 +15743,7 @@
         </is>
       </c>
       <c r="I299" s="2" t="n">
-        <v>558</v>
+        <v>417</v>
       </c>
       <c r="J299" s="4" t="inlineStr">
         <is>
@@ -15794,7 +15794,7 @@
         </is>
       </c>
       <c r="I300" s="2" t="n">
-        <v>515</v>
+        <v>448</v>
       </c>
       <c r="J300" s="4" t="inlineStr">
         <is>
@@ -15845,7 +15845,7 @@
         </is>
       </c>
       <c r="I301" s="2" t="n">
-        <v>516</v>
+        <v>418</v>
       </c>
       <c r="J301" s="4" t="inlineStr">
         <is>
@@ -15896,7 +15896,7 @@
         </is>
       </c>
       <c r="I302" s="2" t="n">
-        <v>1227</v>
+        <v>509</v>
       </c>
       <c r="J302" s="4" t="inlineStr">
         <is>
@@ -15947,7 +15947,7 @@
         </is>
       </c>
       <c r="I303" s="2" t="n">
-        <v>445</v>
+        <v>411</v>
       </c>
       <c r="J303" s="4" t="inlineStr">
         <is>
@@ -15998,7 +15998,7 @@
         </is>
       </c>
       <c r="I304" s="2" t="n">
-        <v>401</v>
+        <v>414</v>
       </c>
       <c r="J304" s="4" t="inlineStr">
         <is>
@@ -16049,7 +16049,7 @@
         </is>
       </c>
       <c r="I305" s="2" t="n">
-        <v>430</v>
+        <v>442</v>
       </c>
       <c r="J305" s="4" t="inlineStr">
         <is>
@@ -16100,7 +16100,7 @@
         </is>
       </c>
       <c r="I306" s="2" t="n">
-        <v>435</v>
+        <v>411</v>
       </c>
       <c r="J306" s="4" t="inlineStr">
         <is>
@@ -16151,7 +16151,7 @@
         </is>
       </c>
       <c r="I307" s="2" t="n">
-        <v>442</v>
+        <v>451</v>
       </c>
       <c r="J307" s="4" t="inlineStr">
         <is>
@@ -16202,7 +16202,7 @@
         </is>
       </c>
       <c r="I308" s="2" t="n">
-        <v>397</v>
+        <v>440</v>
       </c>
       <c r="J308" s="4" t="inlineStr">
         <is>
@@ -16253,7 +16253,7 @@
         </is>
       </c>
       <c r="I309" s="2" t="n">
-        <v>368</v>
+        <v>289</v>
       </c>
       <c r="J309" s="4" t="inlineStr">
         <is>
@@ -16304,7 +16304,7 @@
         </is>
       </c>
       <c r="I310" s="2" t="n">
-        <v>394</v>
+        <v>289</v>
       </c>
       <c r="J310" s="4" t="inlineStr">
         <is>
@@ -16355,7 +16355,7 @@
         </is>
       </c>
       <c r="I311" s="2" t="n">
-        <v>378</v>
+        <v>303</v>
       </c>
       <c r="J311" s="4" t="inlineStr">
         <is>
@@ -16406,7 +16406,7 @@
         </is>
       </c>
       <c r="I312" s="2" t="n">
-        <v>379</v>
+        <v>318</v>
       </c>
       <c r="J312" s="4" t="inlineStr">
         <is>
@@ -16457,7 +16457,7 @@
         </is>
       </c>
       <c r="I313" s="2" t="n">
-        <v>366</v>
+        <v>297</v>
       </c>
       <c r="J313" s="4" t="inlineStr">
         <is>
@@ -16508,7 +16508,7 @@
         </is>
       </c>
       <c r="I314" s="2" t="n">
-        <v>396</v>
+        <v>310</v>
       </c>
       <c r="J314" s="4" t="inlineStr">
         <is>
@@ -16559,7 +16559,7 @@
         </is>
       </c>
       <c r="I315" s="2" t="n">
-        <v>399</v>
+        <v>304</v>
       </c>
       <c r="J315" s="4" t="inlineStr">
         <is>
@@ -16610,7 +16610,7 @@
         </is>
       </c>
       <c r="I316" s="2" t="n">
-        <v>399</v>
+        <v>313</v>
       </c>
       <c r="J316" s="4" t="inlineStr">
         <is>
@@ -16661,7 +16661,7 @@
         </is>
       </c>
       <c r="I317" s="2" t="n">
-        <v>421</v>
+        <v>311</v>
       </c>
       <c r="J317" s="4" t="inlineStr">
         <is>
@@ -16712,7 +16712,7 @@
         </is>
       </c>
       <c r="I318" s="2" t="n">
-        <v>392</v>
+        <v>428</v>
       </c>
       <c r="J318" s="4" t="inlineStr">
         <is>
@@ -16763,7 +16763,7 @@
         </is>
       </c>
       <c r="I319" s="2" t="n">
-        <v>392</v>
+        <v>349</v>
       </c>
       <c r="J319" s="4" t="inlineStr">
         <is>
@@ -16814,7 +16814,7 @@
         </is>
       </c>
       <c r="I320" s="2" t="n">
-        <v>407</v>
+        <v>336</v>
       </c>
       <c r="J320" s="4" t="inlineStr">
         <is>
@@ -16865,7 +16865,7 @@
         </is>
       </c>
       <c r="I321" s="2" t="n">
-        <v>378</v>
+        <v>293</v>
       </c>
       <c r="J321" s="4" t="inlineStr">
         <is>
@@ -16916,7 +16916,7 @@
         </is>
       </c>
       <c r="I322" s="2" t="n">
-        <v>367</v>
+        <v>272</v>
       </c>
       <c r="J322" s="4" t="inlineStr">
         <is>
@@ -16967,7 +16967,7 @@
         </is>
       </c>
       <c r="I323" s="2" t="n">
-        <v>370</v>
+        <v>295</v>
       </c>
       <c r="J323" s="4" t="inlineStr">
         <is>
@@ -17018,7 +17018,7 @@
         </is>
       </c>
       <c r="I324" s="2" t="n">
-        <v>446</v>
+        <v>272</v>
       </c>
       <c r="J324" s="4" t="inlineStr">
         <is>
@@ -17069,7 +17069,7 @@
         </is>
       </c>
       <c r="I325" s="2" t="n">
-        <v>401</v>
+        <v>292</v>
       </c>
       <c r="J325" s="4" t="inlineStr">
         <is>
@@ -17120,7 +17120,7 @@
         </is>
       </c>
       <c r="I326" s="2" t="n">
-        <v>371</v>
+        <v>334</v>
       </c>
       <c r="J326" s="4" t="inlineStr">
         <is>
@@ -17171,7 +17171,7 @@
         </is>
       </c>
       <c r="I327" s="2" t="n">
-        <v>385</v>
+        <v>284</v>
       </c>
       <c r="J327" s="4" t="inlineStr">
         <is>
@@ -17222,7 +17222,7 @@
         </is>
       </c>
       <c r="I328" s="2" t="n">
-        <v>686</v>
+        <v>701</v>
       </c>
       <c r="J328" s="4" t="inlineStr">
         <is>
@@ -17273,7 +17273,7 @@
         </is>
       </c>
       <c r="I329" s="2" t="n">
-        <v>850</v>
+        <v>673</v>
       </c>
       <c r="J329" s="4" t="inlineStr">
         <is>
@@ -17324,7 +17324,7 @@
         </is>
       </c>
       <c r="I330" s="2" t="n">
-        <v>741</v>
+        <v>638</v>
       </c>
       <c r="J330" s="4" t="inlineStr">
         <is>
@@ -17375,7 +17375,7 @@
         </is>
       </c>
       <c r="I331" s="2" t="n">
-        <v>669</v>
+        <v>657</v>
       </c>
       <c r="J331" s="4" t="inlineStr">
         <is>
@@ -17426,7 +17426,7 @@
         </is>
       </c>
       <c r="I332" s="2" t="n">
-        <v>635</v>
+        <v>661</v>
       </c>
       <c r="J332" s="4" t="inlineStr">
         <is>
@@ -17477,7 +17477,7 @@
         </is>
       </c>
       <c r="I333" s="2" t="n">
-        <v>677</v>
+        <v>731</v>
       </c>
       <c r="J333" s="4" t="inlineStr">
         <is>
@@ -17528,7 +17528,7 @@
         </is>
       </c>
       <c r="I334" s="2" t="n">
-        <v>643</v>
+        <v>648</v>
       </c>
       <c r="J334" s="4" t="inlineStr">
         <is>
@@ -17579,7 +17579,7 @@
         </is>
       </c>
       <c r="I335" s="2" t="n">
-        <v>740</v>
+        <v>691</v>
       </c>
       <c r="J335" s="4" t="inlineStr">
         <is>
@@ -17630,7 +17630,7 @@
         </is>
       </c>
       <c r="I336" s="2" t="n">
-        <v>647</v>
+        <v>638</v>
       </c>
       <c r="J336" s="4" t="inlineStr">
         <is>
@@ -17681,7 +17681,7 @@
         </is>
       </c>
       <c r="I337" s="2" t="n">
-        <v>610</v>
+        <v>799</v>
       </c>
       <c r="J337" s="4" t="inlineStr">
         <is>
@@ -17732,7 +17732,7 @@
         </is>
       </c>
       <c r="I338" s="2" t="n">
-        <v>637</v>
+        <v>732</v>
       </c>
       <c r="J338" s="4" t="inlineStr">
         <is>
@@ -17783,7 +17783,7 @@
         </is>
       </c>
       <c r="I339" s="2" t="n">
-        <v>685</v>
+        <v>680</v>
       </c>
       <c r="J339" s="4" t="inlineStr">
         <is>
@@ -17834,7 +17834,7 @@
         </is>
       </c>
       <c r="I340" s="2" t="n">
-        <v>956</v>
+        <v>664</v>
       </c>
       <c r="J340" s="4" t="inlineStr">
         <is>
@@ -17885,7 +17885,7 @@
         </is>
       </c>
       <c r="I341" s="2" t="n">
-        <v>738</v>
+        <v>749</v>
       </c>
       <c r="J341" s="4" t="inlineStr">
         <is>
@@ -17936,7 +17936,7 @@
         </is>
       </c>
       <c r="I342" s="2" t="n">
-        <v>653</v>
+        <v>639</v>
       </c>
       <c r="J342" s="4" t="inlineStr">
         <is>
@@ -17987,7 +17987,7 @@
         </is>
       </c>
       <c r="I343" s="2" t="n">
-        <v>1621</v>
+        <v>713</v>
       </c>
       <c r="J343" s="4" t="inlineStr">
         <is>
@@ -18038,7 +18038,7 @@
         </is>
       </c>
       <c r="I344" s="2" t="n">
-        <v>650</v>
+        <v>662</v>
       </c>
       <c r="J344" s="4" t="inlineStr">
         <is>
@@ -18089,7 +18089,7 @@
         </is>
       </c>
       <c r="I345" s="2" t="n">
-        <v>671</v>
+        <v>796</v>
       </c>
       <c r="J345" s="4" t="inlineStr">
         <is>
@@ -18140,7 +18140,7 @@
         </is>
       </c>
       <c r="I346" s="2" t="n">
-        <v>759</v>
+        <v>653</v>
       </c>
       <c r="J346" s="4" t="inlineStr">
         <is>
@@ -18191,7 +18191,7 @@
         </is>
       </c>
       <c r="I347" s="2" t="n">
-        <v>793</v>
+        <v>755</v>
       </c>
       <c r="J347" s="4" t="inlineStr">
         <is>
@@ -20306,7 +20306,7 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>2026-09-11 11:12:47 UTC</t>
+          <t>2026-09-11 12:50:09 UTC</t>
         </is>
       </c>
     </row>
@@ -20376,7 +20376,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>644 ms</t>
+          <t>597 ms</t>
         </is>
       </c>
     </row>

</xml_diff>